<commit_message>
added comparision question excel table
</commit_message>
<xml_diff>
--- a/test/results/model_comparison/comparison.xlsx
+++ b/test/results/model_comparison/comparison.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leven\PycharmProjects\jogi-agent-clean\test\results\model_comparison\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06E77C3-B8F7-4596-AB18-4E2EBF991AB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF84642-2C52-4042-89B4-B8516CBA0811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{D9DAACF3-2B6D-4249-925C-DCD65B142A30}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{D9DAACF3-2B6D-4249-925C-DCD65B142A30}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="Összefoglaló" sheetId="1" r:id="rId1"/>
+    <sheet name="Kérdések" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="52">
   <si>
     <t>Base Model</t>
   </si>
@@ -79,11 +80,131 @@
   <si>
     <t>Mérés 25 kérdésen történt, csoportonként 3 könnyű, 2 nehéz kérdésen, illetve plusz 5 kombinált kérdésen.</t>
   </si>
+  <si>
+    <t>GDPR rendelet</t>
+  </si>
+  <si>
+    <t>SZJA törvény</t>
+  </si>
+  <si>
+    <t>Kombinált</t>
+  </si>
+  <si>
+    <t>könnyű</t>
+  </si>
+  <si>
+    <t>nehéz</t>
+  </si>
+  <si>
+    <t>összetett</t>
+  </si>
+  <si>
+    <t>Munkavállalóként hány munkanap távollétre vagyok jogosult a hozzátartozóm halála esetén a Munka Törvénykönyve alapján?</t>
+  </si>
+  <si>
+    <t>Legalább hány nappal korábban köteles a munkavállaló írásban bejelenteni a fizetés nélküli szabadság igénybevételét a munkáltatója felé?</t>
+  </si>
+  <si>
+    <t>A munkavállaló súlyos egészségi okból gondozásra szoruló hozzátartozója ápolása céljából évente legfeljebb hány munkanap mentesülésre jogosult a munkavégzési kötelezettsége alól?</t>
+  </si>
+  <si>
+    <t>A felügyeleti hatóság korrekciós hatáskörében eljárva milyen intézkedést hozhat, ha egy adatkezelő adatkezelési tevékenysége megsértette a rendelet rendelkezéseit?</t>
+  </si>
+  <si>
+    <t>Mentesülhet-e az adatkezelő a kártérítési felelősség alól, ha bizonyítani tudja, hogy a kárt előidéző eseményért őt semmilyen módon nem terheli felelősség?</t>
+  </si>
+  <si>
+    <t>Munka Törvénykönyve (Mt,)</t>
+  </si>
+  <si>
+    <t>Egy vállalat átalakulása során (munkáltató személyében bekövetkező változás) az átadó munkáltatónál üzemi tanács nem működik, A munkáltatók megállapodtak, hogy az átvevő munkáltató tájékoztatja a munkavállalókat az átszállásról, Az átvevő munkáltató az átszállás napján írásban közölte a munkáltató azonosító adatait és a munkafeltételek változását, Milyen jogi következménye van annak, hogy a tájékoztatásra az átszállást megelőző 15 napos határidőn belül nem került sor, és milyen felelősségi szabály vonatkozik az átszállás előtti munkavállalói követelésekre?</t>
+  </si>
+  <si>
+    <t>Egy munkavállaló, aki megváltozott munkaképességű, július 1-jén lépett munkaviszonyba, A munkavállaló augusztus hónapban üzemi baleset miatt vált keresőképtelenné, majd a felépülése után, októberben betegség miatt 10 munkanapra keresőképtelenné vált, Jogosult-e az érintett a 120, § szerinti 5 munkanap pótszabadságra az adott naptári évben, és hány munkanap betegszabadság illeti meg az év hátralévő részében a 126, § szabályai alapján?</t>
+  </si>
+  <si>
+    <t>Egy ügyfél vagyoni kárt szenvedett az adatkezelő szabálytalan adatkezelése miatt, Melyik cikk alapján jogosult kártérítést követelni az adatkezelőtől?</t>
+  </si>
+  <si>
+    <t>Egy ügyvédi iroda (adatkezelő) szakmai titoktartási kötelezettség hatálya alá tartozó iratanyagot kezel, A felügyeleti hatóság vizsgálatot indít az irodánál, és betekintést kér az ügyfélaktákba, Hogyan kell a tagállami jog szerinti titoktartási kötelezettséget a 90, cikk alapján összeegyeztetni a felügyeleti hatóság 58, cikk szerinti ellenőrzési hatáskörével, és milyen feltételeknek kell megfelelni ahhoz, hogy a hatóság egyáltalán korlátozhatja az adatkezelőre vonatkozó titoktartási kötelezettséget?</t>
+  </si>
+  <si>
+    <t>Egy érintett a 18, cikk (1) bekezdésének c) pontjára hivatkozva kéri személyes adatai kezelésének korlátozását, mivel az adatkezelőnek a konkrét adatkezelési cél megvalósulása miatt már nincs szüksége az adatokra, de az érintett azokat egy folyamatban lévő polgári peres eljárásban bizonyítékként kívánja felhasználni, Az adatkezelő az adatokat a korlátozást követően egy külső, jogi képviseletet ellátó ügyvédi iroda szerverére kívánja áthelyezni jogi igényeinek védelme érdekében, Megfelel-e ez az adatkezelési művelet a 18, cikk (2) bekezdésének, és milyen tájékoztatási kötelezettségei keletkeznek az adatkezelőnek az adatkezelés esetleges későbbi feloldása kapcsán?</t>
+  </si>
+  <si>
+    <t>Polgári Törvénykönyv (Ptk,)</t>
+  </si>
+  <si>
+    <t>Házastársak elváltak, de nem tudnak megállapodni a közös lakás további használatáról, Melyik szerv dönthet ilyen esetben a lakáshasználat rendezéséről valamelyik fél kérelmére?</t>
+  </si>
+  <si>
+    <t>Egy bank hitelt nyújtott, amelynek biztosítékául két zálogjogosult is bejegyeztetett zálogjogot, Átveheti-e a megelőző ranghelyű zálogjogosult a zálogjog érvényesítését a már megkezdett eljárás során?</t>
+  </si>
+  <si>
+    <t>A vagyonrendelő és a kedvezményezett elégedetlen a vagyonkezelő döntéseivel, ezért írásban utasítják a vagyonkezelőt a kezelt vagyon értékesítésére, Érvényes-e ez az utasítás?</t>
+  </si>
+  <si>
+    <t>Egy határozatlan idejű bérleti szerződés esetén a bérbeadó a hónap 20, napján közli a rendes felmondást a bérlővel, A Ptk, 6:347, § alapján a bérleti jogviszony mikor tekinthető megszűntnek, tekintettel arra, hogy a felek nem a törvényben meghatározott 15, napi határidőt tartották be?</t>
+  </si>
+  <si>
+    <t>Egy vétőképtelen személy kárt okoz egy harmadik félnek, A kártérítési perben a vétőképtelen gondozója bizonyítja, hogy a károkozás idején a felügyeletet megfelelően ellátta, és a nevelésével kapcsolatban semmilyen felróhatóság nem terheli, A Ptk, 6:544, § rendelkezései értelmében mentesül-e a gondozó a kártérítési felelősség alól, vagy a vétőképtelen személy cselekvőképességének hiánya objektív felelősséget von maga után?</t>
+  </si>
+  <si>
+    <t>Egy magánszemély közüzemi szolgáltatója a fogyasztóvédelmi törvényben meghatározott szabályok szerint elengedett egy tartozást, Milyen jövedelemhatár esetén nem keletkezik ebből adóköteles jövedelme a magánszemélynek, ha a kötelezett és a vele közös háztartásban élő hozzátartozóinak egy főre eső jövedelme a nyilatkozattételt megelőző három hónap átlagában a szociális vetítési alap összegének kétszeresét vizsgáljuk?</t>
+  </si>
+  <si>
+    <t>Az SzJA törvény 50, § (7) bekezdése alapján mennyi időre tilos ismételten átalányadózást választania annak az egyéni vállalkozónak, aki az átalányadózását megszüntette, vagy az arra való jogosultsága megszűnt?</t>
+  </si>
+  <si>
+    <t>A 67/C, § alapján az adóévben kriptoeszközzel végrehajtott ügyletből származó ügyleti bevételt akkor nem kell megállapítani, ha az ügyletből származó bevétel a minimálbér mekkora százalékát nem haladja meg, feltéve, hogy a bevétel megszerzésének napján más, azonos tárgyú ügyletből a magánszemély nem szerez bevételt, továbbá az adóévben e bevételek összege a minimálbért nem haladja meg?</t>
+  </si>
+  <si>
+    <t>Egy magánszemély egyéni vállalkozóként mezőgazdasági tevékenységet folytat, és elhatárolt veszteséggel rendelkezik, A vállalkozó az adóév végén megszünteti egyéni vállalkozói jogállását, és tevékenységét mezőgazdasági őstermelőként folytatja tovább, Milyen szabályok szerint számolhatja el a korábbi egyéni vállalkozói időszakból fennmaradt elhatárolt veszteségét az őstermelői jogállás alatt, figyelembe véve a 49/A, § (10) bekezdés d) pontját?</t>
+  </si>
+  <si>
+    <t>A 66, § (1) bekezdés a) pont ae) és ag) alpontja értelmében osztaléknak minősülő juttatások esetében a 66, § (4) bekezdése értelmében mikor nem alkalmazható az osztalékjövedelemre vonatkozó rendelkezés, ha a kedvezményezett magánszemély a jogállását nem alapítói, hanem egyéb, tevékenységnyújtással összefüggő jogcímen szerezte?</t>
+  </si>
+  <si>
+    <t>Egy munkáltató teljesítménybérezési rendszert vezet be, amelyhez a munkavállalók szigorú KPI-jait egy felhőalapú rendszerben tárolja, Az adatvédelmi tisztviselő (GDPR 37, cikk) aggályokat fogalmaz meg a rendszer adatbiztonsága miatt, ugyanakkor a munkáltató a 138, § szerinti teljesítménykövetelmény-megállapítási kötelezettsége kapcsán vitába keveredik a dolgozókkal, Mely jogszabályi rendelkezések alapján kell a munkáltatónak bizonyítania a rendszer jogszerűségét, és milyen adatvédelmi szankciókat kockáztat, ha a teljesítményértékeléshez egészségügyi adatokat (GDPR 9, cikk) is szisztematikusan rögzít?</t>
+  </si>
+  <si>
+    <t>Egy zálogjogosult (Ptk, 5:131, §) el kívánja árverezni egy adós üzemi berendezését, Az eljárás során a zálogjogosult az adós által a cégtől kapott, kedvezményes lakáscélú hitel (SZJA 72, §) dokumentációját is értékesítené, mint a követeléshez kapcsolódó iratanyagot, Hogyan érinti az előzetes értesítési kötelezettség (Ptk, 5:131, §) az adatkezelési szabályokat, ha az értékesítendő iratok az érintettek különleges adatait (GDPR 9, cikk) tartalmazzák, és a zálogtárgy nem esik a gyorsan romló dolgok körébe?</t>
+  </si>
+  <si>
+    <t>Munkáltatói kártérítési felelősség körébe tartozó hiány esetén a felek megállapodnak, hogy a munkavállaló a tartozását a munkáltató által korábban nyújtott munkabérelőleg (SZJA 72, §) elszámolásával egyenlíti ki, A folyamat során azonban a munkáltató a munkavállaló szabadságmegváltását is beszámítaná a hiányba, Milyen munkajogi korlátok vonatkoznak a szabadság kiadására/megváltására (Mt, 115, §) a kártérítési beszámítás során, és hogyan minősül adózási szempontból a kártérítési felelősséggel összefüggő hiány (SZJA 72, § (4) m) pont)?</t>
+  </si>
+  <si>
+    <t>Egy közfeladatot ellátó szerv (GDPR 37, cikk) zálogjogot érvényesít egy olyan ingatlanon, amelynek a tulajdonosa egyúttal a szervnél munkaviszonyban álló magánszemély, A szerv az értékesítési folyamat során a zálogkötelezett munkavállalói jövedelemadatait is kezeli a követelés mértékének megállapításához, Ütközik-e az SZJA törvény 4, § szerinti bevétel fogalma és a munkabér-elszámolás adatkezelési rendje a Ptk, 5:131, § szerinti előzetes értesítési kötelezettséggel, ha a zálogjogosult a közös adatvédelmi tisztviselő révén kívánja biztosítani az adatok védelmét?</t>
+  </si>
+  <si>
+    <t>Biztosítási szerződés keretében a biztosító a fedezetfeltöltés (Ptk, 6:461, §) elmulasztása miatt csökkenti a biztosítási összeget, ugyanakkor az adóhatóság az eredeti (teljes) biztosítási összeg után megfizetett díj kedvezményezettjének jövedelemadózását vizsgálja, Hogyan értelmezhető az SZJA törvény 72, § szerinti kamatkedvezmény, ha a biztosító a fedezetfeltöltés során kedvezményes törlesztési lehetőséget kínál a munkavállaló szerződő félnek, és hogyan kell biztosítani az adatvédelmi tisztviselő bevonását, ha a biztosítási esemény különleges adatot (GDPR 9, cikk) is érint?</t>
+  </si>
+  <si>
+    <t>Question</t>
+  </si>
+  <si>
+    <t>Law</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Error:</t>
+  </si>
+  <si>
+    <t>Error avg.:</t>
+  </si>
+  <si>
+    <t>Avg.:</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="167" formatCode="0.000"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -101,7 +222,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -109,13 +230,345 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -189,7 +642,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Feuil1!$A$2</c:f>
+              <c:f>Összefoglaló!$A$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -210,7 +663,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Feuil1!$B$1:$E$1</c:f>
+              <c:f>Összefoglaló!$B$1:$E$1</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -230,7 +683,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Feuil1!$B$2:$E$2</c:f>
+              <c:f>Összefoglaló!$B$2:$E$2</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -510,7 +963,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Feuil1!$B$1:$E$1</c:f>
+              <c:f>Összefoglaló!$B$1:$E$1</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -530,7 +983,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Feuil1!$B$3:$E$3</c:f>
+              <c:f>Összefoglaló!$B$3:$E$3</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
@@ -810,7 +1263,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Feuil1!$B$1:$E$1</c:f>
+              <c:f>Összefoglaló!$B$1:$E$1</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -830,7 +1283,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Feuil1!$B$4:$E$4</c:f>
+              <c:f>Összefoglaló!$B$4:$E$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -1092,7 +1545,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-UM"/>
+          <a:endParaRPr lang="de-DE"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1118,7 +1571,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Feuil1!$B$1:$E$1</c:f>
+              <c:f>Összefoglaló!$B$1:$E$1</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -1138,7 +1591,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Feuil1!$B$5:$E$5</c:f>
+              <c:f>Összefoglaló!$B$5:$E$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -1433,7 +1886,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Feuil1!$B$1:$E$1</c:f>
+              <c:f>Összefoglaló!$B$1:$E$1</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -1453,7 +1906,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Feuil1!$B$6:$E$6</c:f>
+              <c:f>Összefoglaló!$B$6:$E$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -1744,7 +2197,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Feuil1!$B$1:$E$1</c:f>
+              <c:f>Összefoglaló!$B$1:$E$1</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -1764,7 +2217,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Feuil1!$B$7:$E$7</c:f>
+              <c:f>Összefoglaló!$B$7:$E$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -6003,4 +6456,1473 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F36BC549-5F0D-4260-974E-C5029CF103D9}">
+  <dimension ref="A1:O30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="16.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="3"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="3"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K1" s="3"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="N1" s="3"/>
+      <c r="O1" s="4"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="34" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="35" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="36" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="K2" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="L2" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="M2" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="N2" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="O2" s="20" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="22">
+        <v>1</v>
+      </c>
+      <c r="E3" s="23">
+        <v>1</v>
+      </c>
+      <c r="F3" s="24">
+        <v>1</v>
+      </c>
+      <c r="G3" s="22">
+        <v>1</v>
+      </c>
+      <c r="H3" s="23">
+        <v>0.94117647058823495</v>
+      </c>
+      <c r="I3" s="24">
+        <v>0.66666666666666596</v>
+      </c>
+      <c r="J3" s="22">
+        <v>1</v>
+      </c>
+      <c r="K3" s="23">
+        <v>1</v>
+      </c>
+      <c r="L3" s="24">
+        <v>0.66666666666666596</v>
+      </c>
+      <c r="M3" s="22">
+        <v>1</v>
+      </c>
+      <c r="N3" s="23">
+        <v>0.9375</v>
+      </c>
+      <c r="O3" s="25">
+        <v>0.66666666666666596</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="6">
+        <v>0.76923076923076905</v>
+      </c>
+      <c r="E4" s="7">
+        <v>1</v>
+      </c>
+      <c r="F4" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="G4" s="6">
+        <v>0.91666666666666596</v>
+      </c>
+      <c r="H4" s="7">
+        <v>1</v>
+      </c>
+      <c r="I4" s="8">
+        <v>0.66666666666666596</v>
+      </c>
+      <c r="J4" s="6">
+        <v>1</v>
+      </c>
+      <c r="K4" s="7">
+        <v>1</v>
+      </c>
+      <c r="L4" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="M4" s="6">
+        <v>1</v>
+      </c>
+      <c r="N4" s="7">
+        <v>0.92307692307692302</v>
+      </c>
+      <c r="O4" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="6">
+        <v>1</v>
+      </c>
+      <c r="E5" s="7">
+        <v>1</v>
+      </c>
+      <c r="F5" s="8">
+        <v>0.66666666666666596</v>
+      </c>
+      <c r="G5" s="6">
+        <v>1</v>
+      </c>
+      <c r="H5" s="7">
+        <v>0.8125</v>
+      </c>
+      <c r="I5" s="8">
+        <v>0.66666666666666596</v>
+      </c>
+      <c r="J5" s="6">
+        <v>1</v>
+      </c>
+      <c r="K5" s="7">
+        <v>0.95652173913043403</v>
+      </c>
+      <c r="L5" s="8">
+        <v>0.6</v>
+      </c>
+      <c r="M5" s="6">
+        <v>0.93333333333333302</v>
+      </c>
+      <c r="N5" s="7">
+        <v>1</v>
+      </c>
+      <c r="O5" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="6">
+        <v>1</v>
+      </c>
+      <c r="E6" s="7">
+        <v>0.94444444444444398</v>
+      </c>
+      <c r="F6" s="8">
+        <v>1</v>
+      </c>
+      <c r="G6" s="6">
+        <v>1</v>
+      </c>
+      <c r="H6" s="7">
+        <v>1</v>
+      </c>
+      <c r="I6" s="8">
+        <v>1</v>
+      </c>
+      <c r="J6" s="6">
+        <v>1</v>
+      </c>
+      <c r="K6" s="7">
+        <v>1</v>
+      </c>
+      <c r="L6" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="M6" s="6">
+        <v>1</v>
+      </c>
+      <c r="N6" s="7">
+        <v>1</v>
+      </c>
+      <c r="O6" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="9">
+        <v>1</v>
+      </c>
+      <c r="E7" s="10">
+        <v>1</v>
+      </c>
+      <c r="F7" s="11">
+        <v>1</v>
+      </c>
+      <c r="G7" s="9">
+        <v>1</v>
+      </c>
+      <c r="H7" s="10">
+        <v>1</v>
+      </c>
+      <c r="I7" s="11">
+        <v>1</v>
+      </c>
+      <c r="J7" s="9">
+        <v>1</v>
+      </c>
+      <c r="K7" s="10">
+        <v>0.92</v>
+      </c>
+      <c r="L7" s="11">
+        <v>1</v>
+      </c>
+      <c r="M7" s="9">
+        <v>1</v>
+      </c>
+      <c r="N7" s="10">
+        <v>0.83333333333333304</v>
+      </c>
+      <c r="O7" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="22">
+        <v>1</v>
+      </c>
+      <c r="E8" s="23">
+        <v>1</v>
+      </c>
+      <c r="F8" s="24">
+        <v>1</v>
+      </c>
+      <c r="G8" s="22">
+        <v>0.91666666666666596</v>
+      </c>
+      <c r="H8" s="23">
+        <v>1</v>
+      </c>
+      <c r="I8" s="24">
+        <v>0.75</v>
+      </c>
+      <c r="J8" s="22">
+        <v>1</v>
+      </c>
+      <c r="K8" s="23">
+        <v>1</v>
+      </c>
+      <c r="L8" s="24">
+        <v>0.75</v>
+      </c>
+      <c r="M8" s="22">
+        <v>1</v>
+      </c>
+      <c r="N8" s="23">
+        <v>1</v>
+      </c>
+      <c r="O8" s="25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="6">
+        <v>1</v>
+      </c>
+      <c r="E9" s="7">
+        <v>0.95</v>
+      </c>
+      <c r="F9" s="8">
+        <v>1</v>
+      </c>
+      <c r="G9" s="6">
+        <v>1</v>
+      </c>
+      <c r="H9" s="7">
+        <v>1</v>
+      </c>
+      <c r="I9" s="8">
+        <v>1</v>
+      </c>
+      <c r="J9" s="6">
+        <v>1</v>
+      </c>
+      <c r="K9" s="7">
+        <v>0.83333333333333304</v>
+      </c>
+      <c r="L9" s="8">
+        <v>1</v>
+      </c>
+      <c r="M9" s="6">
+        <v>1</v>
+      </c>
+      <c r="N9" s="7">
+        <v>0.95833333333333304</v>
+      </c>
+      <c r="O9" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="6">
+        <v>1</v>
+      </c>
+      <c r="E10" s="7">
+        <v>1</v>
+      </c>
+      <c r="F10" s="8">
+        <v>1</v>
+      </c>
+      <c r="G10" s="6">
+        <v>1</v>
+      </c>
+      <c r="H10" s="7">
+        <v>1</v>
+      </c>
+      <c r="I10" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="J10" s="6">
+        <v>1</v>
+      </c>
+      <c r="K10" s="7">
+        <v>1</v>
+      </c>
+      <c r="L10" s="8">
+        <v>1</v>
+      </c>
+      <c r="M10" s="6">
+        <v>1</v>
+      </c>
+      <c r="N10" s="7">
+        <v>1</v>
+      </c>
+      <c r="O10" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="6">
+        <v>1</v>
+      </c>
+      <c r="E11" s="7">
+        <v>1</v>
+      </c>
+      <c r="F11" s="8">
+        <v>1</v>
+      </c>
+      <c r="G11" s="6">
+        <v>1</v>
+      </c>
+      <c r="H11" s="7">
+        <v>1</v>
+      </c>
+      <c r="I11" s="8">
+        <v>1</v>
+      </c>
+      <c r="J11" s="6">
+        <v>1</v>
+      </c>
+      <c r="K11" s="7">
+        <v>1</v>
+      </c>
+      <c r="L11" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="M11" s="6">
+        <v>1</v>
+      </c>
+      <c r="N11" s="7">
+        <v>1</v>
+      </c>
+      <c r="O11" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="9">
+        <v>1</v>
+      </c>
+      <c r="E12" s="10">
+        <v>0.94736842105263097</v>
+      </c>
+      <c r="F12" s="11">
+        <v>1</v>
+      </c>
+      <c r="G12" s="9">
+        <v>1</v>
+      </c>
+      <c r="H12" s="10">
+        <v>0.95652173913043403</v>
+      </c>
+      <c r="I12" s="11">
+        <v>0.75</v>
+      </c>
+      <c r="J12" s="9">
+        <v>1</v>
+      </c>
+      <c r="K12" s="10">
+        <v>0.95</v>
+      </c>
+      <c r="L12" s="11">
+        <v>1</v>
+      </c>
+      <c r="M12" s="9">
+        <v>1</v>
+      </c>
+      <c r="N12" s="10">
+        <v>1</v>
+      </c>
+      <c r="O12" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="22">
+        <v>1</v>
+      </c>
+      <c r="E13" s="23">
+        <v>1</v>
+      </c>
+      <c r="F13" s="24">
+        <v>1</v>
+      </c>
+      <c r="G13" s="22">
+        <v>1</v>
+      </c>
+      <c r="H13" s="23">
+        <v>1</v>
+      </c>
+      <c r="I13" s="24">
+        <v>1</v>
+      </c>
+      <c r="J13" s="22">
+        <v>1</v>
+      </c>
+      <c r="K13" s="23">
+        <v>1</v>
+      </c>
+      <c r="L13" s="24">
+        <v>1</v>
+      </c>
+      <c r="M13" s="22">
+        <v>1</v>
+      </c>
+      <c r="N13" s="23">
+        <v>1</v>
+      </c>
+      <c r="O13" s="25">
+        <v>0.66666666666666596</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="6">
+        <v>1</v>
+      </c>
+      <c r="E14" s="7">
+        <v>1</v>
+      </c>
+      <c r="F14" s="8">
+        <v>1</v>
+      </c>
+      <c r="G14" s="6">
+        <v>1</v>
+      </c>
+      <c r="H14" s="7">
+        <v>1</v>
+      </c>
+      <c r="I14" s="8">
+        <v>1</v>
+      </c>
+      <c r="J14" s="6">
+        <v>1</v>
+      </c>
+      <c r="K14" s="7">
+        <v>1</v>
+      </c>
+      <c r="L14" s="8">
+        <v>1</v>
+      </c>
+      <c r="M14" s="6">
+        <v>1</v>
+      </c>
+      <c r="N14" s="7">
+        <v>1</v>
+      </c>
+      <c r="O14" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D15" s="6">
+        <v>1</v>
+      </c>
+      <c r="E15" s="7">
+        <v>1</v>
+      </c>
+      <c r="F15" s="8">
+        <v>1</v>
+      </c>
+      <c r="G15" s="6">
+        <v>1</v>
+      </c>
+      <c r="H15" s="7">
+        <v>1</v>
+      </c>
+      <c r="I15" s="8">
+        <v>1</v>
+      </c>
+      <c r="J15" s="6">
+        <v>1</v>
+      </c>
+      <c r="K15" s="7">
+        <v>1</v>
+      </c>
+      <c r="L15" s="8">
+        <v>0.72727272727272696</v>
+      </c>
+      <c r="M15" s="6">
+        <v>1</v>
+      </c>
+      <c r="N15" s="7">
+        <v>1</v>
+      </c>
+      <c r="O15" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" s="6">
+        <v>1</v>
+      </c>
+      <c r="E16" s="7">
+        <v>1</v>
+      </c>
+      <c r="F16" s="8">
+        <v>1</v>
+      </c>
+      <c r="G16" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="H16" s="7">
+        <v>0.88888888888888795</v>
+      </c>
+      <c r="I16" s="8">
+        <v>1</v>
+      </c>
+      <c r="J16" s="6">
+        <v>0.90909090909090895</v>
+      </c>
+      <c r="K16" s="7">
+        <v>1</v>
+      </c>
+      <c r="L16" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="M16" s="6">
+        <v>1</v>
+      </c>
+      <c r="N16" s="7">
+        <v>1</v>
+      </c>
+      <c r="O16" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="28" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="D17" s="9">
+        <v>1</v>
+      </c>
+      <c r="E17" s="10">
+        <v>1</v>
+      </c>
+      <c r="F17" s="11">
+        <v>1</v>
+      </c>
+      <c r="G17" s="9">
+        <v>1</v>
+      </c>
+      <c r="H17" s="10">
+        <v>0.95454545454545403</v>
+      </c>
+      <c r="I17" s="11">
+        <v>1</v>
+      </c>
+      <c r="J17" s="9">
+        <v>0.94117647058823495</v>
+      </c>
+      <c r="K17" s="10">
+        <v>0.952380952380952</v>
+      </c>
+      <c r="L17" s="11">
+        <v>1</v>
+      </c>
+      <c r="M17" s="9">
+        <v>1</v>
+      </c>
+      <c r="N17" s="10">
+        <v>1</v>
+      </c>
+      <c r="O17" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="22">
+        <v>1</v>
+      </c>
+      <c r="E18" s="23">
+        <v>1</v>
+      </c>
+      <c r="F18" s="24">
+        <v>1</v>
+      </c>
+      <c r="G18" s="22">
+        <v>1</v>
+      </c>
+      <c r="H18" s="23">
+        <v>0.90909090909090895</v>
+      </c>
+      <c r="I18" s="24">
+        <v>1</v>
+      </c>
+      <c r="J18" s="22">
+        <v>1</v>
+      </c>
+      <c r="K18" s="23">
+        <v>0.92307692307692302</v>
+      </c>
+      <c r="L18" s="24">
+        <v>1</v>
+      </c>
+      <c r="M18" s="22">
+        <v>1</v>
+      </c>
+      <c r="N18" s="23">
+        <v>1</v>
+      </c>
+      <c r="O18" s="25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" s="6">
+        <v>0.9375</v>
+      </c>
+      <c r="E19" s="7">
+        <v>0.94117647058823495</v>
+      </c>
+      <c r="F19" s="8">
+        <v>1</v>
+      </c>
+      <c r="G19" s="6">
+        <v>1</v>
+      </c>
+      <c r="H19" s="7">
+        <v>0.64285714285714202</v>
+      </c>
+      <c r="I19" s="8">
+        <v>1</v>
+      </c>
+      <c r="J19" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="K19" s="7">
+        <v>1</v>
+      </c>
+      <c r="L19" s="8">
+        <v>1</v>
+      </c>
+      <c r="M19" s="6">
+        <v>1</v>
+      </c>
+      <c r="N19" s="7">
+        <v>1</v>
+      </c>
+      <c r="O19" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D20" s="6">
+        <v>0.91666666666666596</v>
+      </c>
+      <c r="E20" s="7">
+        <v>1</v>
+      </c>
+      <c r="F20" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="G20" s="6">
+        <v>1</v>
+      </c>
+      <c r="H20" s="7">
+        <v>1</v>
+      </c>
+      <c r="I20" s="8">
+        <v>0.66666666666666596</v>
+      </c>
+      <c r="J20" s="6">
+        <v>1</v>
+      </c>
+      <c r="K20" s="7">
+        <v>1</v>
+      </c>
+      <c r="L20" s="8">
+        <v>0.66666666666666596</v>
+      </c>
+      <c r="M20" s="6">
+        <v>1</v>
+      </c>
+      <c r="N20" s="7">
+        <v>1</v>
+      </c>
+      <c r="O20" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="6">
+        <v>0.94444444444444398</v>
+      </c>
+      <c r="E21" s="7">
+        <v>1</v>
+      </c>
+      <c r="F21" s="8">
+        <v>1</v>
+      </c>
+      <c r="G21" s="6">
+        <v>1</v>
+      </c>
+      <c r="H21" s="7">
+        <v>1</v>
+      </c>
+      <c r="I21" s="8">
+        <v>1</v>
+      </c>
+      <c r="J21" s="6">
+        <v>1</v>
+      </c>
+      <c r="K21" s="7">
+        <v>1</v>
+      </c>
+      <c r="L21" s="8">
+        <v>1</v>
+      </c>
+      <c r="M21" s="6">
+        <v>0.90909090909090895</v>
+      </c>
+      <c r="N21" s="7">
+        <v>1</v>
+      </c>
+      <c r="O21" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="D22" s="9">
+        <v>1</v>
+      </c>
+      <c r="E22" s="10">
+        <v>1</v>
+      </c>
+      <c r="F22" s="11">
+        <v>1</v>
+      </c>
+      <c r="G22" s="9">
+        <v>1</v>
+      </c>
+      <c r="H22" s="10">
+        <v>1</v>
+      </c>
+      <c r="I22" s="11">
+        <v>0.8</v>
+      </c>
+      <c r="J22" s="9">
+        <v>1</v>
+      </c>
+      <c r="K22" s="10">
+        <v>1</v>
+      </c>
+      <c r="L22" s="11">
+        <v>1</v>
+      </c>
+      <c r="M22" s="9">
+        <v>0.93333333333333302</v>
+      </c>
+      <c r="N22" s="10">
+        <v>1</v>
+      </c>
+      <c r="O22" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="D23" s="22">
+        <v>1</v>
+      </c>
+      <c r="E23" s="23">
+        <v>1</v>
+      </c>
+      <c r="F23" s="24">
+        <v>1</v>
+      </c>
+      <c r="G23" s="22">
+        <v>1</v>
+      </c>
+      <c r="H23" s="23">
+        <v>1</v>
+      </c>
+      <c r="I23" s="24">
+        <v>1</v>
+      </c>
+      <c r="J23" s="22">
+        <v>1</v>
+      </c>
+      <c r="K23" s="23">
+        <v>1</v>
+      </c>
+      <c r="L23" s="24">
+        <v>1</v>
+      </c>
+      <c r="M23" s="22">
+        <v>1</v>
+      </c>
+      <c r="N23" s="23">
+        <v>1</v>
+      </c>
+      <c r="O23" s="25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" s="6">
+        <v>0.86666666666666603</v>
+      </c>
+      <c r="E24" s="7">
+        <v>0.95</v>
+      </c>
+      <c r="F24" s="8">
+        <v>1</v>
+      </c>
+      <c r="G24" s="6">
+        <v>1</v>
+      </c>
+      <c r="H24" s="7">
+        <v>1</v>
+      </c>
+      <c r="I24" s="8">
+        <v>1</v>
+      </c>
+      <c r="J24" s="6">
+        <v>1</v>
+      </c>
+      <c r="K24" s="7">
+        <v>1</v>
+      </c>
+      <c r="L24" s="8">
+        <v>1</v>
+      </c>
+      <c r="M24" s="6">
+        <v>1</v>
+      </c>
+      <c r="N24" s="7">
+        <v>0.95454545454545403</v>
+      </c>
+      <c r="O24" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25" s="6">
+        <v>1</v>
+      </c>
+      <c r="E25" s="7">
+        <v>0.94736842105263097</v>
+      </c>
+      <c r="F25" s="8">
+        <v>1</v>
+      </c>
+      <c r="G25" s="6">
+        <v>1</v>
+      </c>
+      <c r="H25" s="7">
+        <v>1</v>
+      </c>
+      <c r="I25" s="8">
+        <v>1</v>
+      </c>
+      <c r="J25" s="6">
+        <v>1</v>
+      </c>
+      <c r="K25" s="7">
+        <v>1</v>
+      </c>
+      <c r="L25" s="8">
+        <v>1</v>
+      </c>
+      <c r="M25" s="6">
+        <v>1</v>
+      </c>
+      <c r="N25" s="7">
+        <v>1</v>
+      </c>
+      <c r="O25" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D26" s="6">
+        <v>1</v>
+      </c>
+      <c r="E26" s="7">
+        <v>1</v>
+      </c>
+      <c r="F26" s="8">
+        <v>1</v>
+      </c>
+      <c r="G26" s="6">
+        <v>1</v>
+      </c>
+      <c r="H26" s="7">
+        <v>1</v>
+      </c>
+      <c r="I26" s="8">
+        <v>1</v>
+      </c>
+      <c r="J26" s="6">
+        <v>1</v>
+      </c>
+      <c r="K26" s="7">
+        <v>1</v>
+      </c>
+      <c r="L26" s="8">
+        <v>0.85714285714285698</v>
+      </c>
+      <c r="M26" s="6">
+        <v>1</v>
+      </c>
+      <c r="N26" s="7">
+        <v>1</v>
+      </c>
+      <c r="O26" s="27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="B27" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="D27" s="9">
+        <v>0.86666666666666603</v>
+      </c>
+      <c r="E27" s="10">
+        <v>1</v>
+      </c>
+      <c r="F27" s="11">
+        <v>1</v>
+      </c>
+      <c r="G27" s="9">
+        <v>1</v>
+      </c>
+      <c r="H27" s="10">
+        <v>0.952380952380952</v>
+      </c>
+      <c r="I27" s="11">
+        <v>1</v>
+      </c>
+      <c r="J27" s="9">
+        <v>1</v>
+      </c>
+      <c r="K27" s="10">
+        <v>1</v>
+      </c>
+      <c r="L27" s="11">
+        <v>1</v>
+      </c>
+      <c r="M27" s="9">
+        <v>1</v>
+      </c>
+      <c r="N27" s="10">
+        <v>0.90909090909090895</v>
+      </c>
+      <c r="O27" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C28" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="D28" s="12">
+        <f>AVERAGE(D3:D27)</f>
+        <v>0.97204700854700843</v>
+      </c>
+      <c r="E28" s="13">
+        <f t="shared" ref="E28:O28" si="0">AVERAGE(E3:E27)</f>
+        <v>0.98721431028551765</v>
+      </c>
+      <c r="F28" s="14">
+        <f t="shared" si="0"/>
+        <v>0.96666666666666656</v>
+      </c>
+      <c r="G28" s="12">
+        <f t="shared" si="0"/>
+        <v>0.98533333333333328</v>
+      </c>
+      <c r="H28" s="13">
+        <f t="shared" si="0"/>
+        <v>0.96231846229928053</v>
+      </c>
+      <c r="I28" s="14">
+        <f t="shared" si="0"/>
+        <v>0.90866666666666662</v>
+      </c>
+      <c r="J28" s="12">
+        <f t="shared" si="0"/>
+        <v>0.98601069518716566</v>
+      </c>
+      <c r="K28" s="13">
+        <f t="shared" si="0"/>
+        <v>0.98141251791686568</v>
+      </c>
+      <c r="L28" s="14">
+        <f t="shared" si="0"/>
+        <v>0.88470995670995667</v>
+      </c>
+      <c r="M28" s="12">
+        <f t="shared" si="0"/>
+        <v>0.99103030303030304</v>
+      </c>
+      <c r="N28" s="13">
+        <f t="shared" si="0"/>
+        <v>0.98063519813519806</v>
+      </c>
+      <c r="O28" s="14">
+        <f t="shared" si="0"/>
+        <v>0.97333333333333327</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="C29" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="D29" s="15">
+        <f>25-COUNTIF(D3:D27,1)</f>
+        <v>6</v>
+      </c>
+      <c r="E29" s="16">
+        <f t="shared" ref="E29:F29" si="1">25-COUNTIF(E3:E27,1)</f>
+        <v>6</v>
+      </c>
+      <c r="F29" s="17">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="G29" s="15">
+        <f>25-COUNTIF(G3:G27,1)</f>
+        <v>3</v>
+      </c>
+      <c r="H29" s="16">
+        <f t="shared" ref="H29:I29" si="2">25-COUNTIF(H3:H27,1)</f>
+        <v>8</v>
+      </c>
+      <c r="I29" s="17">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="J29" s="15">
+        <f>25-COUNTIF(J3:J27,1)</f>
+        <v>3</v>
+      </c>
+      <c r="K29" s="16">
+        <f t="shared" ref="K29:L29" si="3">25-COUNTIF(K3:K27,1)</f>
+        <v>6</v>
+      </c>
+      <c r="L29" s="17">
+        <f t="shared" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="M29" s="15">
+        <f>25-COUNTIF(M3:M27,1)</f>
+        <v>3</v>
+      </c>
+      <c r="N29" s="16">
+        <f t="shared" ref="N29:O29" si="4">25-COUNTIF(N3:N27,1)</f>
+        <v>6</v>
+      </c>
+      <c r="O29" s="17">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="C30" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="D30" s="31">
+        <f>AVERAGE(D29:F29)</f>
+        <v>5</v>
+      </c>
+      <c r="E30" s="32"/>
+      <c r="F30" s="33"/>
+      <c r="G30" s="31">
+        <f>AVERAGE(G29:I29)</f>
+        <v>6.333333333333333</v>
+      </c>
+      <c r="H30" s="32"/>
+      <c r="I30" s="33"/>
+      <c r="J30" s="31">
+        <f>AVERAGE(J29:L29)</f>
+        <v>6.333333333333333</v>
+      </c>
+      <c r="K30" s="32"/>
+      <c r="L30" s="33"/>
+      <c r="M30" s="31">
+        <f>AVERAGE(M29:O29)</f>
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="N30" s="32"/>
+      <c r="O30" s="33"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="J1:L1"/>
+    <mergeCell ref="M1:O1"/>
+    <mergeCell ref="D30:F30"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="J30:L30"/>
+    <mergeCell ref="M30:O30"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D3:O28">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D28:O28">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D29:O29">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{1CBD6AED-E61C-4CA0-8210-5EA7351ABED4}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{1CBD6AED-E61C-4CA0-8210-5EA7351ABED4}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D29:O29</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>